<commit_message>
Update Raw_data.xlsx — added Apr 2026
</commit_message>
<xml_diff>
--- a/data/Raw_data.xlsx
+++ b/data/Raw_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bharatmimmani/Documents/TATA STEEL/TS/dashboard/HRC_Pipeline/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A1ADDF6-F8EF-4346-9C55-55EF7BDA8353}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0830A60B-DC60-CB4F-929D-838AF6A010F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15780" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14380" yWindow="620" windowWidth="14420" windowHeight="15880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -171,15 +171,20 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -202,9 +207,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -633,8 +639,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:J124"/>
+  <dimension ref="A1:J125"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="17" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -693,8 +702,8 @@
       <c r="H2">
         <v>99.61</v>
       </c>
-      <c r="I2">
-        <v>1.93</v>
+      <c r="I2" s="2">
+        <v>2.0853000000000002</v>
       </c>
       <c r="J2">
         <v>373</v>
@@ -725,8 +734,8 @@
       <c r="H3">
         <v>98.21</v>
       </c>
-      <c r="I3">
-        <v>1.79</v>
+      <c r="I3" s="2">
+        <v>1.7795000000000001</v>
       </c>
       <c r="J3">
         <v>290</v>
@@ -757,8 +766,8 @@
       <c r="H4">
         <v>94.59</v>
       </c>
-      <c r="I4">
-        <v>1.84</v>
+      <c r="I4" s="2">
+        <v>1.8891</v>
       </c>
       <c r="J4">
         <v>370</v>
@@ -789,8 +798,8 @@
       <c r="H5">
         <v>93.08</v>
       </c>
-      <c r="I5">
-        <v>1.83</v>
+      <c r="I5" s="2">
+        <v>1.8051999999999999</v>
       </c>
       <c r="J5">
         <v>515</v>
@@ -821,8 +830,8 @@
       <c r="H6">
         <v>95.89</v>
       </c>
-      <c r="I6">
-        <v>1.82</v>
+      <c r="I6" s="2">
+        <v>1.8062</v>
       </c>
       <c r="J6">
         <v>681</v>
@@ -853,8 +862,8 @@
       <c r="H7">
         <v>96.14</v>
       </c>
-      <c r="I7">
-        <v>1.67</v>
+      <c r="I7" s="2">
+        <v>1.6440999999999999</v>
       </c>
       <c r="J7">
         <v>626</v>
@@ -885,8 +894,8 @@
       <c r="H8">
         <v>95.53</v>
       </c>
-      <c r="I8">
-        <v>1.66</v>
+      <c r="I8" s="2">
+        <v>1.504</v>
       </c>
       <c r="J8">
         <v>669</v>
@@ -917,8 +926,8 @@
       <c r="H9">
         <v>96.02</v>
       </c>
-      <c r="I9">
-        <v>1.67</v>
+      <c r="I9" s="2">
+        <v>1.5553999999999999</v>
       </c>
       <c r="J9">
         <v>730</v>
@@ -949,8 +958,8 @@
       <c r="H10">
         <v>95.46</v>
       </c>
-      <c r="I10">
-        <v>1.72</v>
+      <c r="I10" s="2">
+        <v>1.6248</v>
       </c>
       <c r="J10">
         <v>921</v>
@@ -981,8 +990,8 @@
       <c r="H11">
         <v>98.45</v>
       </c>
-      <c r="I11">
-        <v>1.78</v>
+      <c r="I11" s="2">
+        <v>1.7539</v>
       </c>
       <c r="J11">
         <v>921</v>
@@ -1013,8 +1022,8 @@
       <c r="H12">
         <v>101.5</v>
       </c>
-      <c r="I12">
-        <v>2.1</v>
+      <c r="I12" s="2">
+        <v>2.1493000000000002</v>
       </c>
       <c r="J12">
         <v>1108</v>
@@ -1045,8 +1054,8 @@
       <c r="H13">
         <v>102.39</v>
       </c>
-      <c r="I13">
-        <v>2.25</v>
+      <c r="I13" s="2">
+        <v>2.4897999999999998</v>
       </c>
       <c r="J13">
         <v>961</v>
@@ -1077,8 +1086,8 @@
       <c r="H14">
         <v>99.51</v>
       </c>
-      <c r="I14">
-        <v>2.4</v>
+      <c r="I14" s="2">
+        <v>2.4253999999999998</v>
       </c>
       <c r="J14">
         <v>1049</v>
@@ -1109,8 +1118,8 @@
       <c r="H15">
         <v>101.12</v>
       </c>
-      <c r="I15">
-        <v>2.39</v>
+      <c r="I15" s="2">
+        <v>2.4150999999999998</v>
       </c>
       <c r="J15">
         <v>1084</v>
@@ -1141,8 +1150,8 @@
       <c r="H16">
         <v>100.35</v>
       </c>
-      <c r="I16">
-        <v>2.42</v>
+      <c r="I16" s="2">
+        <v>2.4790999999999999</v>
       </c>
       <c r="J16">
         <v>1261</v>
@@ -1173,8 +1182,8 @@
       <c r="H17">
         <v>99.05</v>
       </c>
-      <c r="I17">
-        <v>2.2799999999999998</v>
+      <c r="I17" s="2">
+        <v>2.2854999999999999</v>
       </c>
       <c r="J17">
         <v>1342</v>
@@ -1205,8 +1214,8 @@
       <c r="H18">
         <v>96.92</v>
       </c>
-      <c r="I18">
-        <v>2.27</v>
+      <c r="I18" s="2">
+        <v>2.2970999999999999</v>
       </c>
       <c r="J18">
         <v>1245</v>
@@ -1237,8 +1246,8 @@
       <c r="H19">
         <v>95.66</v>
       </c>
-      <c r="I19">
-        <v>2.2400000000000002</v>
+      <c r="I19" s="2">
+        <v>2.1846999999999999</v>
       </c>
       <c r="J19">
         <v>1044</v>
@@ -1269,8 +1278,8 @@
       <c r="H20">
         <v>92.86</v>
       </c>
-      <c r="I20">
-        <v>2.2999999999999998</v>
+      <c r="I20" s="2">
+        <v>2.3149000000000002</v>
       </c>
       <c r="J20">
         <v>1127</v>
@@ -1301,8 +1310,8 @@
       <c r="H21">
         <v>92.67</v>
       </c>
-      <c r="I21">
-        <v>2.23</v>
+      <c r="I21" s="2">
+        <v>2.2044999999999999</v>
       </c>
       <c r="J21">
         <v>1167</v>
@@ -1333,8 +1342,8 @@
       <c r="H22">
         <v>93.08</v>
       </c>
-      <c r="I22">
-        <v>2.29</v>
+      <c r="I22" s="2">
+        <v>2.1968000000000001</v>
       </c>
       <c r="J22">
         <v>1485</v>
@@ -1365,8 +1374,8 @@
       <c r="H23">
         <v>94.55</v>
       </c>
-      <c r="I23">
-        <v>2.37</v>
+      <c r="I23" s="2">
+        <v>2.3561999999999999</v>
       </c>
       <c r="J23">
         <v>1506</v>
@@ -1397,8 +1406,8 @@
       <c r="H24">
         <v>93.01</v>
       </c>
-      <c r="I24">
-        <v>2.34</v>
+      <c r="I24" s="2">
+        <v>2.3530000000000002</v>
       </c>
       <c r="J24">
         <v>1506</v>
@@ -1429,8 +1438,8 @@
       <c r="H25">
         <v>92.12</v>
       </c>
-      <c r="I25">
-        <v>2.38</v>
+      <c r="I25" s="2">
+        <v>2.4062000000000001</v>
       </c>
       <c r="J25">
         <v>1366</v>
@@ -1461,8 +1470,8 @@
       <c r="H26">
         <v>89.13</v>
       </c>
-      <c r="I26">
-        <v>2.75</v>
+      <c r="I26" s="2">
+        <v>2.5821000000000001</v>
       </c>
       <c r="J26">
         <v>1366</v>
@@ -1493,8 +1502,8 @@
       <c r="H27">
         <v>90.61</v>
       </c>
-      <c r="I27">
-        <v>2.89</v>
+      <c r="I27" s="2">
+        <v>2.8597000000000001</v>
       </c>
       <c r="J27">
         <v>1182</v>
@@ -1525,8 +1534,8 @@
       <c r="H28">
         <v>89.97</v>
       </c>
-      <c r="I28">
-        <v>2.84</v>
+      <c r="I28" s="2">
+        <v>2.8422000000000001</v>
       </c>
       <c r="J28">
         <v>1096</v>
@@ -1557,8 +1566,8 @@
       <c r="H29">
         <v>91.84</v>
       </c>
-      <c r="I29">
-        <v>2.91</v>
+      <c r="I29" s="2">
+        <v>2.8690000000000002</v>
       </c>
       <c r="J29">
         <v>1244</v>
@@ -1589,8 +1598,8 @@
       <c r="H30">
         <v>93.99</v>
       </c>
-      <c r="I30">
-        <v>2.95</v>
+      <c r="I30" s="2">
+        <v>2.9777</v>
       </c>
       <c r="J30">
         <v>1274</v>
@@ -1621,8 +1630,8 @@
       <c r="H31">
         <v>94.63</v>
       </c>
-      <c r="I31">
-        <v>2.9</v>
+      <c r="I31" s="2">
+        <v>2.9123999999999999</v>
       </c>
       <c r="J31">
         <v>1547</v>
@@ -1653,8 +1662,8 @@
       <c r="H32">
         <v>94.49</v>
       </c>
-      <c r="I32">
-        <v>2.93</v>
+      <c r="I32" s="2">
+        <v>2.8889999999999998</v>
       </c>
       <c r="J32">
         <v>1667</v>
@@ -1685,8 +1694,8 @@
       <c r="H33">
         <v>95.14</v>
       </c>
-      <c r="I33">
-        <v>2.87</v>
+      <c r="I33" s="2">
+        <v>2.8891</v>
       </c>
       <c r="J33">
         <v>1524</v>
@@ -1717,8 +1726,8 @@
       <c r="H34">
         <v>95.19</v>
       </c>
-      <c r="I34">
-        <v>2.99</v>
+      <c r="I34" s="2">
+        <v>3.0042</v>
       </c>
       <c r="J34">
         <v>1471</v>
@@ -1749,8 +1758,8 @@
       <c r="H35">
         <v>97.13</v>
       </c>
-      <c r="I35">
-        <v>3.05</v>
+      <c r="I35" s="2">
+        <v>3.1522999999999999</v>
       </c>
       <c r="J35">
         <v>1541</v>
@@ -1781,8 +1790,8 @@
       <c r="H36">
         <v>97.27</v>
       </c>
-      <c r="I36">
-        <v>3</v>
+      <c r="I36" s="2">
+        <v>3.117</v>
       </c>
       <c r="J36">
         <v>1303</v>
@@ -1813,8 +1822,8 @@
       <c r="H37">
         <v>96.17</v>
       </c>
-      <c r="I37">
-        <v>2.83</v>
+      <c r="I37" s="2">
+        <v>2.8325999999999998</v>
       </c>
       <c r="J37">
         <v>1271</v>
@@ -1845,8 +1854,8 @@
       <c r="H38">
         <v>95.58</v>
       </c>
-      <c r="I38">
-        <v>2.54</v>
+      <c r="I38" s="2">
+        <v>2.7138</v>
       </c>
       <c r="J38">
         <v>1282</v>
@@ -1877,8 +1886,8 @@
       <c r="H39">
         <v>96.16</v>
       </c>
-      <c r="I39">
-        <v>2.46</v>
+      <c r="I39" s="2">
+        <v>2.6762999999999999</v>
       </c>
       <c r="J39">
         <v>920</v>
@@ -1909,8 +1918,8 @@
       <c r="H40">
         <v>97.28</v>
       </c>
-      <c r="I40">
-        <v>2.33</v>
+      <c r="I40" s="2">
+        <v>2.5710000000000002</v>
       </c>
       <c r="J40">
         <v>770</v>
@@ -1941,8 +1950,8 @@
       <c r="H41">
         <v>97.48</v>
       </c>
-      <c r="I41">
-        <v>2.37</v>
+      <c r="I41" s="2">
+        <v>2.5324</v>
       </c>
       <c r="J41">
         <v>972</v>
@@ -1973,8 +1982,8 @@
       <c r="H42">
         <v>97.75</v>
       </c>
-      <c r="I42">
-        <v>2.25</v>
+      <c r="I42" s="2">
+        <v>2.395</v>
       </c>
       <c r="J42">
         <v>1009</v>
@@ -2005,8 +2014,8 @@
       <c r="H43">
         <v>96.13</v>
       </c>
-      <c r="I43">
-        <v>2.0699999999999998</v>
+      <c r="I43" s="2">
+        <v>2.0739999999999998</v>
       </c>
       <c r="J43">
         <v>1097</v>
@@ -2037,8 +2046,8 @@
       <c r="H44">
         <v>98.52</v>
       </c>
-      <c r="I44">
-        <v>2.12</v>
+      <c r="I44" s="2">
+        <v>2.0590999999999999</v>
       </c>
       <c r="J44">
         <v>1858</v>
@@ -2069,8 +2078,8 @@
       <c r="H45">
         <v>98.92</v>
       </c>
-      <c r="I45">
-        <v>1.82</v>
+      <c r="I45" s="2">
+        <v>1.6264000000000001</v>
       </c>
       <c r="J45">
         <v>2073</v>
@@ -2101,8 +2110,8 @@
       <c r="H46">
         <v>99.38</v>
       </c>
-      <c r="I46">
-        <v>1.88</v>
+      <c r="I46" s="2">
+        <v>1.6995</v>
       </c>
       <c r="J46">
         <v>2318</v>
@@ -2133,8 +2142,8 @@
       <c r="H47">
         <v>97.35</v>
       </c>
-      <c r="I47">
-        <v>1.92</v>
+      <c r="I47" s="2">
+        <v>1.7068000000000001</v>
       </c>
       <c r="J47">
         <v>1796</v>
@@ -2165,8 +2174,8 @@
       <c r="H48">
         <v>98.27</v>
       </c>
-      <c r="I48">
-        <v>1.98</v>
+      <c r="I48" s="2">
+        <v>1.8121</v>
       </c>
       <c r="J48">
         <v>1322</v>
@@ -2197,8 +2206,8 @@
       <c r="H49">
         <v>96.39</v>
       </c>
-      <c r="I49">
-        <v>2.0099999999999998</v>
+      <c r="I49" s="2">
+        <v>1.8629</v>
       </c>
       <c r="J49">
         <v>1090</v>
@@ -2229,8 +2238,8 @@
       <c r="H50">
         <v>97.39</v>
       </c>
-      <c r="I50">
-        <v>1.38</v>
+      <c r="I50" s="2">
+        <v>1.7576000000000001</v>
       </c>
       <c r="J50">
         <v>713</v>
@@ -2261,8 +2270,8 @@
       <c r="H51">
         <v>98.13</v>
       </c>
-      <c r="I51">
-        <v>1.2</v>
+      <c r="I51" s="2">
+        <v>1.5042</v>
       </c>
       <c r="J51">
         <v>469</v>
@@ -2293,8 +2302,8 @@
       <c r="H52">
         <v>99.05</v>
       </c>
-      <c r="I52">
-        <v>0.91</v>
+      <c r="I52" s="2">
+        <v>0.87</v>
       </c>
       <c r="J52">
         <v>557</v>
@@ -2325,8 +2334,8 @@
       <c r="H53">
         <v>99.02</v>
       </c>
-      <c r="I53">
-        <v>0.73</v>
+      <c r="I53" s="2">
+        <v>0.65759999999999996</v>
       </c>
       <c r="J53">
         <v>718</v>
@@ -2357,8 +2366,8 @@
       <c r="H54">
         <v>98.34</v>
       </c>
-      <c r="I54">
-        <v>0.76</v>
+      <c r="I54" s="2">
+        <v>0.67400000000000004</v>
       </c>
       <c r="J54">
         <v>504</v>
@@ -2389,8 +2398,8 @@
       <c r="H55">
         <v>97.39</v>
       </c>
-      <c r="I55">
-        <v>0.8</v>
+      <c r="I55" s="2">
+        <v>0.72860000000000003</v>
       </c>
       <c r="J55">
         <v>1746</v>
@@ -2421,8 +2430,8 @@
       <c r="H56">
         <v>93.49</v>
       </c>
-      <c r="I56">
-        <v>0.73</v>
+      <c r="I56" s="2">
+        <v>0.62360000000000004</v>
       </c>
       <c r="J56">
         <v>1820</v>
@@ -2453,8 +2462,8 @@
       <c r="H57">
         <v>92.14</v>
       </c>
-      <c r="I57">
-        <v>0.77</v>
+      <c r="I57" s="2">
+        <v>0.65</v>
       </c>
       <c r="J57">
         <v>1370</v>
@@ -2485,8 +2494,8 @@
       <c r="H58">
         <v>93.89</v>
       </c>
-      <c r="I58">
-        <v>0.76</v>
+      <c r="I58" s="2">
+        <v>0.67949999999999999</v>
       </c>
       <c r="J58">
         <v>1660</v>
@@ -2517,8 +2526,8 @@
       <c r="H59">
         <v>94.04</v>
       </c>
-      <c r="I59">
-        <v>0.87</v>
+      <c r="I59" s="2">
+        <v>0.78710000000000002</v>
       </c>
       <c r="J59">
         <v>1681</v>
@@ -2549,8 +2558,8 @@
       <c r="H60">
         <v>91.87</v>
       </c>
-      <c r="I60">
-        <v>0.86</v>
+      <c r="I60" s="2">
+        <v>0.87</v>
       </c>
       <c r="J60">
         <v>1407</v>
@@ -2581,8 +2590,8 @@
       <c r="H61">
         <v>89.94</v>
       </c>
-      <c r="I61">
-        <v>0.93</v>
+      <c r="I61" s="2">
+        <v>0.93359999999999999</v>
       </c>
       <c r="J61">
         <v>1384</v>
@@ -2613,8 +2622,8 @@
       <c r="H62">
         <v>90.58</v>
       </c>
-      <c r="I62">
-        <v>1.25</v>
+      <c r="I62" s="2">
+        <v>1.0810999999999999</v>
       </c>
       <c r="J62">
         <v>1592</v>
@@ -2645,8 +2654,8 @@
       <c r="H63">
         <v>90.93</v>
       </c>
-      <c r="I63">
-        <v>1.39</v>
+      <c r="I63" s="2">
+        <v>1.2579</v>
       </c>
       <c r="J63">
         <v>1607</v>
@@ -2677,8 +2686,8 @@
       <c r="H64">
         <v>93.23</v>
       </c>
-      <c r="I64">
-        <v>1.58</v>
+      <c r="I64" s="2">
+        <v>1.6109</v>
       </c>
       <c r="J64">
         <v>1966</v>
@@ -2709,8 +2718,8 @@
       <c r="H65">
         <v>91.28</v>
       </c>
-      <c r="I65">
-        <v>1.52</v>
+      <c r="I65" s="2">
+        <v>1.635</v>
       </c>
       <c r="J65">
         <v>2491</v>
@@ -2741,8 +2750,8 @@
       <c r="H66">
         <v>89.84</v>
       </c>
-      <c r="I66">
-        <v>1.54</v>
+      <c r="I66" s="2">
+        <v>1.621</v>
       </c>
       <c r="J66">
         <v>2814</v>
@@ -2773,8 +2782,8 @@
       <c r="H67">
         <v>92.44</v>
       </c>
-      <c r="I67">
-        <v>1.47</v>
+      <c r="I67" s="2">
+        <v>1.5190999999999999</v>
       </c>
       <c r="J67">
         <v>3214</v>
@@ -2805,8 +2814,8 @@
       <c r="H68">
         <v>92.17</v>
       </c>
-      <c r="I68">
-        <v>1.35</v>
+      <c r="I68" s="2">
+        <v>1.3186</v>
       </c>
       <c r="J68">
         <v>3230</v>
@@ -2837,8 +2846,8 @@
       <c r="H69">
         <v>92.63</v>
       </c>
-      <c r="I69">
-        <v>1.35</v>
+      <c r="I69" s="2">
+        <v>1.2831999999999999</v>
       </c>
       <c r="J69">
         <v>3291</v>
@@ -2869,8 +2878,8 @@
       <c r="H70">
         <v>94.25</v>
       </c>
-      <c r="I70">
-        <v>1.41</v>
+      <c r="I70" s="2">
+        <v>1.3748</v>
       </c>
       <c r="J70">
         <v>4383</v>
@@ -2901,8 +2910,8 @@
       <c r="H71">
         <v>94.12</v>
       </c>
-      <c r="I71">
-        <v>1.54</v>
+      <c r="I71" s="2">
+        <v>1.5825</v>
       </c>
       <c r="J71">
         <v>5650</v>
@@ -2933,8 +2942,8 @@
       <c r="H72">
         <v>95.99</v>
       </c>
-      <c r="I72">
-        <v>1.51</v>
+      <c r="I72" s="2">
+        <v>1.5595000000000001</v>
       </c>
       <c r="J72">
         <v>3295</v>
@@ -2965,8 +2974,8 @@
       <c r="H73">
         <v>95.67</v>
       </c>
-      <c r="I73">
-        <v>1.47</v>
+      <c r="I73" s="2">
+        <v>1.4650000000000001</v>
       </c>
       <c r="J73">
         <v>2217</v>
@@ -2997,8 +3006,8 @@
       <c r="H74">
         <v>96.54</v>
       </c>
-      <c r="I74">
-        <v>2.2200000000000002</v>
+      <c r="I74" s="2">
+        <v>1.764</v>
       </c>
       <c r="J74">
         <v>2217</v>
@@ -3029,8 +3038,8 @@
       <c r="H75">
         <v>96.71</v>
       </c>
-      <c r="I75">
-        <v>2.38</v>
+      <c r="I75" s="2">
+        <v>1.9341999999999999</v>
       </c>
       <c r="J75">
         <v>2196</v>
@@ -3061,8 +3070,8 @@
       <c r="H76">
         <v>98.31</v>
       </c>
-      <c r="I76">
-        <v>2.4500000000000002</v>
+      <c r="I76" s="2">
+        <v>2.1278000000000001</v>
       </c>
       <c r="J76">
         <v>2500</v>
@@ -3093,8 +3102,8 @@
       <c r="H77">
         <v>102.96</v>
       </c>
-      <c r="I77">
-        <v>2.76</v>
+      <c r="I77" s="2">
+        <v>2.7475000000000001</v>
       </c>
       <c r="J77">
         <v>2708</v>
@@ -3125,8 +3134,8 @@
       <c r="H78">
         <v>101.75</v>
       </c>
-      <c r="I78">
-        <v>2.86</v>
+      <c r="I78" s="2">
+        <v>2.8980999999999999</v>
       </c>
       <c r="J78">
         <v>2805</v>
@@ -3157,8 +3166,8 @@
       <c r="H79">
         <v>104.69</v>
       </c>
-      <c r="I79">
-        <v>3.15</v>
+      <c r="I79" s="2">
+        <v>3.1433</v>
       </c>
       <c r="J79">
         <v>2421</v>
@@ -3189,8 +3198,8 @@
       <c r="H80">
         <v>105.9</v>
       </c>
-      <c r="I80">
-        <v>2.88</v>
+      <c r="I80" s="2">
+        <v>2.8959999999999999</v>
       </c>
       <c r="J80">
         <v>2165</v>
@@ -3221,8 +3230,8 @@
       <c r="H81">
         <v>108.7</v>
       </c>
-      <c r="I81">
-        <v>2.97</v>
+      <c r="I81" s="2">
+        <v>2.8978000000000002</v>
       </c>
       <c r="J81">
         <v>1991</v>
@@ -3253,8 +3262,8 @@
       <c r="H82">
         <v>112.12</v>
       </c>
-      <c r="I82">
-        <v>3.39</v>
+      <c r="I82" s="2">
+        <v>3.5190000000000001</v>
       </c>
       <c r="J82">
         <v>1762</v>
@@ -3285,8 +3294,8 @@
       <c r="H83">
         <v>111.53</v>
       </c>
-      <c r="I83">
-        <v>3.58</v>
+      <c r="I83" s="2">
+        <v>3.9834999999999998</v>
       </c>
       <c r="J83">
         <v>1533</v>
@@ -3317,8 +3326,8 @@
       <c r="H84">
         <v>105.95</v>
       </c>
-      <c r="I84">
-        <v>3.31</v>
+      <c r="I84" s="2">
+        <v>3.891</v>
       </c>
       <c r="J84">
         <v>1297</v>
@@ -3349,8 +3358,8 @@
       <c r="H85">
         <v>103.52</v>
       </c>
-      <c r="I85">
-        <v>3.41</v>
+      <c r="I85" s="2">
+        <v>3.6162000000000001</v>
       </c>
       <c r="J85">
         <v>1515</v>
@@ -3381,8 +3390,8 @@
       <c r="H86">
         <v>102.1</v>
       </c>
-      <c r="I86">
-        <v>3.68</v>
+      <c r="I86" s="2">
+        <v>3.5314999999999999</v>
       </c>
       <c r="J86">
         <v>1515</v>
@@ -3413,8 +3422,8 @@
       <c r="H87">
         <v>104.87</v>
       </c>
-      <c r="I87">
-        <v>3.92</v>
+      <c r="I87" s="2">
+        <v>3.7467999999999999</v>
       </c>
       <c r="J87">
         <v>889</v>
@@ -3445,8 +3454,8 @@
       <c r="H88">
         <v>102.51</v>
       </c>
-      <c r="I88">
-        <v>3.67</v>
+      <c r="I88" s="2">
+        <v>3.6629999999999998</v>
       </c>
       <c r="J88">
         <v>1282</v>
@@ -3477,8 +3486,8 @@
       <c r="H89">
         <v>101.67</v>
       </c>
-      <c r="I89">
-        <v>3.65</v>
+      <c r="I89" s="2">
+        <v>3.46</v>
       </c>
       <c r="J89">
         <v>1505</v>
@@ -3509,8 +3518,8 @@
       <c r="H90">
         <v>104.32</v>
       </c>
-      <c r="I90">
-        <v>3.77</v>
+      <c r="I90" s="2">
+        <v>3.5735999999999999</v>
       </c>
       <c r="J90">
         <v>1200</v>
@@ -3541,8 +3550,8 @@
       <c r="H91">
         <v>102.91</v>
       </c>
-      <c r="I91">
-        <v>3.87</v>
+      <c r="I91" s="2">
+        <v>3.7481</v>
       </c>
       <c r="J91">
         <v>1045</v>
@@ -3573,8 +3582,8 @@
       <c r="H92">
         <v>101.86</v>
       </c>
-      <c r="I92">
-        <v>3.92</v>
+      <c r="I92" s="2">
+        <v>3.8995000000000002</v>
       </c>
       <c r="J92">
         <v>1078</v>
@@ -3605,8 +3614,8 @@
       <c r="H93">
         <v>103.62</v>
       </c>
-      <c r="I93">
-        <v>4.1399999999999997</v>
+      <c r="I93" s="2">
+        <v>4.1677999999999997</v>
       </c>
       <c r="J93">
         <v>1280</v>
@@ -3637,8 +3646,8 @@
       <c r="H94">
         <v>106.17</v>
       </c>
-      <c r="I94">
-        <v>4.24</v>
+      <c r="I94" s="2">
+        <v>4.3789999999999996</v>
       </c>
       <c r="J94">
         <v>1500</v>
@@ -3669,8 +3678,8 @@
       <c r="H95">
         <v>106.66</v>
       </c>
-      <c r="I95">
-        <v>4.47</v>
+      <c r="I95" s="2">
+        <v>4.7980999999999998</v>
       </c>
       <c r="J95">
         <v>1800</v>
@@ -3701,8 +3710,8 @@
       <c r="H96">
         <v>103.5</v>
       </c>
-      <c r="I96">
-        <v>4.25</v>
+      <c r="I96" s="2">
+        <v>4.5029000000000003</v>
       </c>
       <c r="J96">
         <v>2095</v>
@@ -3733,8 +3742,8 @@
       <c r="H97">
         <v>101.33</v>
       </c>
-      <c r="I97">
-        <v>3.89</v>
+      <c r="I97" s="2">
+        <v>4.0199999999999996</v>
       </c>
       <c r="J97">
         <v>2094</v>
@@ -3765,8 +3774,8 @@
       <c r="H98">
         <v>103.27</v>
       </c>
-      <c r="I98">
-        <v>4.1500000000000004</v>
+      <c r="I98" s="2">
+        <v>4.0580999999999996</v>
       </c>
       <c r="J98">
         <v>2094</v>
@@ -3797,8 +3806,8 @@
       <c r="H99">
         <v>104.16</v>
       </c>
-      <c r="I99">
-        <v>4.2300000000000004</v>
+      <c r="I99" s="2">
+        <v>4.2074999999999996</v>
       </c>
       <c r="J99">
         <v>1724</v>
@@ -3829,8 +3838,8 @@
       <c r="H100">
         <v>104.55</v>
       </c>
-      <c r="I100">
-        <v>4.2300000000000004</v>
+      <c r="I100" s="2">
+        <v>4.2084999999999999</v>
       </c>
       <c r="J100">
         <v>2109</v>
@@ -3861,8 +3870,8 @@
       <c r="H101">
         <v>106.22</v>
       </c>
-      <c r="I101">
-        <v>4.4400000000000004</v>
+      <c r="I101" s="2">
+        <v>4.5391000000000004</v>
       </c>
       <c r="J101">
         <v>1800</v>
@@ -3893,8 +3902,8 @@
       <c r="H102">
         <v>104.67</v>
       </c>
-      <c r="I102">
-        <v>4.32</v>
+      <c r="I102" s="2">
+        <v>4.4823000000000004</v>
       </c>
       <c r="J102">
         <v>1713</v>
@@ -3925,8 +3934,8 @@
       <c r="H103">
         <v>105.87</v>
       </c>
-      <c r="I103">
-        <v>4.21</v>
+      <c r="I103" s="2">
+        <v>4.3052999999999999</v>
       </c>
       <c r="J103">
         <v>1737</v>
@@ -3957,8 +3966,8 @@
       <c r="H104">
         <v>104.1</v>
       </c>
-      <c r="I104">
-        <v>4.2</v>
+      <c r="I104" s="2">
+        <v>4.2485999999999997</v>
       </c>
       <c r="J104">
         <v>1952</v>
@@ -3989,8 +3998,8 @@
       <c r="H105">
         <v>101.7</v>
       </c>
-      <c r="I105">
-        <v>3.99</v>
+      <c r="I105" s="2">
+        <v>3.8708999999999998</v>
       </c>
       <c r="J105">
         <v>1726</v>
@@ -4021,8 +4030,8 @@
       <c r="H106">
         <v>100.78</v>
       </c>
-      <c r="I106">
-        <v>3.9</v>
+      <c r="I106" s="2">
+        <v>3.7235</v>
       </c>
       <c r="J106">
         <v>2065</v>
@@ -4053,8 +4062,8 @@
       <c r="H107">
         <v>103.98</v>
       </c>
-      <c r="I107">
-        <v>4.2</v>
+      <c r="I107" s="2">
+        <v>4.0955000000000004</v>
       </c>
       <c r="J107">
         <v>1754</v>
@@ -4085,8 +4094,8 @@
       <c r="H108">
         <v>105.74</v>
       </c>
-      <c r="I108">
-        <v>4.28</v>
+      <c r="I108" s="2">
+        <v>4.3558000000000003</v>
       </c>
       <c r="J108">
         <v>1361</v>
@@ -4117,8 +4126,8 @@
       <c r="H109">
         <v>108.49</v>
       </c>
-      <c r="I109">
-        <v>4.3600000000000003</v>
+      <c r="I109" s="2">
+        <v>4.3914</v>
       </c>
       <c r="J109">
         <v>997</v>
@@ -4149,8 +4158,8 @@
       <c r="H110">
         <v>108.37</v>
       </c>
-      <c r="I110">
-        <v>4.49</v>
+      <c r="I110" s="2">
+        <v>4.6289999999999996</v>
       </c>
       <c r="J110">
         <v>1100</v>
@@ -4181,8 +4190,8 @@
       <c r="H111">
         <v>107.61</v>
       </c>
-      <c r="I111">
-        <v>4.3600000000000003</v>
+      <c r="I111" s="2">
+        <v>4.4511000000000003</v>
       </c>
       <c r="J111">
         <v>985</v>
@@ -4213,8 +4222,8 @@
       <c r="H112">
         <v>104.21</v>
       </c>
-      <c r="I112">
-        <v>4.28</v>
+      <c r="I112" s="2">
+        <v>4.2805</v>
       </c>
       <c r="J112">
         <v>1261</v>
@@ -4245,8 +4254,8 @@
       <c r="H113">
         <v>99.47</v>
       </c>
-      <c r="I113">
-        <v>4.28</v>
+      <c r="I113" s="2">
+        <v>4.2789999999999999</v>
       </c>
       <c r="J113">
         <v>1283</v>
@@ -4277,8 +4286,8 @@
       <c r="H114">
         <v>99.33</v>
       </c>
-      <c r="I114">
-        <v>4.4000000000000004</v>
+      <c r="I114" s="2">
+        <v>4.4238</v>
       </c>
       <c r="J114">
         <v>1400</v>
@@ -4309,8 +4318,8 @@
       <c r="H115">
         <v>96.88</v>
       </c>
-      <c r="I115">
-        <v>4.34</v>
+      <c r="I115" s="2">
+        <v>4.3834999999999997</v>
       </c>
       <c r="J115">
         <v>1500</v>
@@ -4341,8 +4350,8 @@
       <c r="H116">
         <v>100.03</v>
       </c>
-      <c r="I116">
-        <v>4.37</v>
+      <c r="I116" s="2">
+        <v>4.3917999999999999</v>
       </c>
       <c r="J116">
         <v>1650</v>
@@ -4373,8 +4382,8 @@
       <c r="H117">
         <v>97.77</v>
       </c>
-      <c r="I117">
-        <v>4.28</v>
+      <c r="I117" s="2">
+        <v>4.2648000000000001</v>
       </c>
       <c r="J117">
         <v>1800</v>
@@ -4405,8 +4414,8 @@
       <c r="H118">
         <v>97.77</v>
       </c>
-      <c r="I118">
-        <v>4.21</v>
+      <c r="I118" s="2">
+        <v>4.1204999999999998</v>
       </c>
       <c r="J118">
         <v>2100</v>
@@ -4437,8 +4446,8 @@
       <c r="H119">
         <v>99.8</v>
       </c>
-      <c r="I119">
-        <v>4.1399999999999997</v>
+      <c r="I119" s="2">
+        <v>4.0617999999999999</v>
       </c>
       <c r="J119">
         <v>2400</v>
@@ -4469,8 +4478,8 @@
       <c r="H120">
         <v>99.46</v>
       </c>
-      <c r="I120">
-        <v>4.18</v>
+      <c r="I120" s="2">
+        <v>4.0938999999999997</v>
       </c>
       <c r="J120">
         <v>2814</v>
@@ -4501,8 +4510,8 @@
       <c r="H121">
         <v>98.28</v>
       </c>
-      <c r="I121">
-        <v>4.21</v>
+      <c r="I121" s="2">
+        <v>4.1432000000000002</v>
       </c>
       <c r="J121">
         <v>1877</v>
@@ -4533,8 +4542,8 @@
       <c r="H122">
         <v>96.99</v>
       </c>
-      <c r="I122">
-        <v>4.24</v>
+      <c r="I122" s="2">
+        <v>4.2134999999999998</v>
       </c>
       <c r="J122">
         <v>2050</v>
@@ -4557,7 +4566,7 @@
         <v>67.92</v>
       </c>
       <c r="F123">
-        <v>617.77599999999995</v>
+        <v>611.55700000000002</v>
       </c>
       <c r="G123">
         <v>49</v>
@@ -4565,8 +4574,8 @@
       <c r="H123">
         <v>97.61</v>
       </c>
-      <c r="I123">
-        <v>4.09</v>
+      <c r="I123" s="2">
+        <v>4.1257999999999999</v>
       </c>
       <c r="J123">
         <v>1950</v>
@@ -4586,10 +4595,10 @@
         <v>220.25</v>
       </c>
       <c r="E124">
-        <v>94.06</v>
+        <v>102.86</v>
       </c>
       <c r="F124">
-        <v>549.31308333333334</v>
+        <v>615.95500000000004</v>
       </c>
       <c r="G124">
         <v>50.4</v>
@@ -4597,11 +4606,43 @@
       <c r="H124">
         <v>99.96</v>
       </c>
-      <c r="I124">
-        <v>4.3</v>
+      <c r="I124" s="2">
+        <v>4.2458999999999998</v>
       </c>
       <c r="J124">
         <v>2100</v>
+      </c>
+    </row>
+    <row r="125" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A125" s="1">
+        <v>46113</v>
+      </c>
+      <c r="B125">
+        <v>500</v>
+      </c>
+      <c r="C125">
+        <v>107</v>
+      </c>
+      <c r="D125">
+        <v>233.05</v>
+      </c>
+      <c r="E125">
+        <v>108.64</v>
+      </c>
+      <c r="F125">
+        <v>595</v>
+      </c>
+      <c r="G125">
+        <v>50</v>
+      </c>
+      <c r="H125">
+        <v>98.08</v>
+      </c>
+      <c r="I125" s="2">
+        <v>4.3190999999999997</v>
+      </c>
+      <c r="J125">
+        <v>2400</v>
       </c>
     </row>
   </sheetData>

</xml_diff>